<commit_message>
Add tests for label auditing and markdown rendering
- Implemented comprehensive tests for the label audit process in `test_labelaudit.py`, ensuring that citations are verified against the printed figures and that various edge cases are handled correctly.
- Created tests in `test_pagemd.py` to validate the markdown rendering of financial statements, focusing on the correct reconstruction of split numbers and the proper identification of current periods in tables.
- Both test files utilize existing financial reports to ensure accuracy and reliability of the tests.
</commit_message>
<xml_diff>
--- a/data/ground_truth/ADMR.xlsx
+++ b/data/ground_truth/ADMR.xlsx
@@ -603,8 +603,10 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>1</v>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>ADMR</t>
+        </is>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>

</xml_diff>